<commit_message>
- minor changes in the design: GND PGND connection, added layer for DC+ at im828, labels to LEDs - added comments in schematics - added some excel files that are useful for commissioning (adc conversion factors, dutycyc to temperature)
</commit_message>
<xml_diff>
--- a/docs/IM828_kritIC_Liste.xlsx
+++ b/docs/IM828_kritIC_Liste.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_sic_inverter_828xcc\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E5EC8A2-25E6-4B9A-9994-CFE1318F875D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA15C847-1FC4-49FC-A358-BF85BEEBA983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{37F19541-0A2A-42C3-BD89-660E50FCB47F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Herstellernr</t>
   </si>
@@ -90,6 +90,39 @@
   </si>
   <si>
     <t>NXJ2S0505MC</t>
+  </si>
+  <si>
+    <t>LQM31PN4R7M00L</t>
+  </si>
+  <si>
+    <t>B32778Z</t>
+  </si>
+  <si>
+    <t>2220Y6300105KXTWS2</t>
+  </si>
+  <si>
+    <t>LM358DR</t>
+  </si>
+  <si>
+    <t>TC7SZ86FU,LJ(CT</t>
+  </si>
+  <si>
+    <t>T2N7002AK,LM</t>
+  </si>
+  <si>
+    <t>LTV-356T</t>
+  </si>
+  <si>
+    <t>4mm Buchse bk</t>
+  </si>
+  <si>
+    <t>17 bestellt wegen phase fault pcb</t>
+  </si>
+  <si>
+    <t>4mm Buchse bl</t>
+  </si>
+  <si>
+    <t>4mm Buchse rd</t>
   </si>
 </sst>
 </file>
@@ -440,7 +473,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -448,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E48B796E-366E-458A-B05D-DECE29806BFC}">
-  <dimension ref="A2:D12"/>
+  <dimension ref="A2:F25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.26953125" bestFit="1" customWidth="1"/>
@@ -493,7 +526,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="1">
-        <f t="shared" ref="D5:D12" si="0">5*C5</f>
+        <f t="shared" ref="D5:D10" si="0">5*C5</f>
         <v>5</v>
       </c>
     </row>
@@ -558,33 +591,164 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="0"/>
-        <v>5</v>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1">
+        <f>5*C12</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <f t="shared" ref="D13:D25" si="1">5*C13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15">
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>